<commit_message>
Completed AdmissionGPT with ML, RAG, Gemini and Streamlit chatbot
</commit_message>
<xml_diff>
--- a/data/faq.xlsx
+++ b/data/faq.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Internship\AdmissionGPT\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C96382A-5D9B-4919-84A5-419898B30D0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6522AE4C-CA74-4394-A5A6-D9D1D49E641A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" xr2:uid="{8D7A6797-B82E-4FBA-A02D-FDB479BAFB40}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="108">
   <si>
     <t>Question</t>
   </si>
@@ -36,91 +36,319 @@
     <t>What is KEAM?</t>
   </si>
   <si>
-    <t>Kerala Engineering Architecture and Medical entrance examination conducted by CEE Kerala.</t>
-  </si>
-  <si>
-    <t>What is MEC?</t>
-  </si>
-  <si>
-    <t>Government Model Engineering College is one of Kerala's premier engineering colleges.</t>
-  </si>
-  <si>
-    <t>What is CSE?</t>
-  </si>
-  <si>
-    <t>Computer Science and Engineering.</t>
-  </si>
-  <si>
-    <t>What is CSBS?</t>
-  </si>
-  <si>
-    <t>Computer Science and Business Systems.</t>
-  </si>
-  <si>
-    <t>What is ECE?</t>
-  </si>
-  <si>
-    <t>Electronics and Communication Engineering.</t>
-  </si>
-  <si>
-    <t>What is EEE?</t>
-  </si>
-  <si>
-    <t>Electrical and Electronics Engineering.</t>
-  </si>
-  <si>
-    <t>What is VLSI?</t>
-  </si>
-  <si>
-    <t>Electronics Engineering specializing in VLSI Design.</t>
-  </si>
-  <si>
-    <t>What is Biomedical Engineering?</t>
-  </si>
-  <si>
-    <t>Electronics and Biomedical Engineering combines electronics and healthcare technologies.</t>
-  </si>
-  <si>
-    <t>Which branch has best placements?</t>
-  </si>
-  <si>
-    <t>Generally CSE and CSBS have the highest placement opportunities.</t>
-  </si>
-  <si>
-    <t>Is MEC a government college?</t>
-  </si>
-  <si>
-    <t>Yes, MEC is a government-controlled institution under IHRD.</t>
-  </si>
-  <si>
-    <t>Where is MEC located?</t>
-  </si>
-  <si>
-    <t>Thrikkakara, Kochi, Kerala.</t>
-  </si>
-  <si>
-    <t>How many branches are available in MEC?</t>
-  </si>
-  <si>
-    <t>MEC offers CSE, CSBS, ECE, EEE, VLSI, Biomedical and Mechanical Engineering.</t>
-  </si>
-  <si>
-    <t>What can you do?</t>
-  </si>
-  <si>
-    <t>I can predict branch preferences, analyze admission chances and answer MEC-related questions.</t>
-  </si>
-  <si>
-    <t>How do I use AdmissionGPT?</t>
-  </si>
-  <si>
-    <t>Enter your KEAM rank and category to get admission analysis.</t>
-  </si>
-  <si>
-    <t>Can you predict my branch?</t>
-  </si>
-  <si>
-    <t>Yes, provide your KEAM rank and category.</t>
+    <t>What is Computer Science &amp; Engineering?</t>
+  </si>
+  <si>
+    <t>Computer Science &amp; Engineering (CSE) focuses on programming, software development, artificial intelligence, data structures, operating systems, databases, networking, and computer architecture.</t>
+  </si>
+  <si>
+    <t>What is Computer Science and Business Systems?</t>
+  </si>
+  <si>
+    <t>Computer Science and Business Systems (CSBS) combines core computer science subjects with business analytics, management, finance, and entrepreneurship.</t>
+  </si>
+  <si>
+    <t>What is Electronics &amp; Communication Engineering?</t>
+  </si>
+  <si>
+    <t>Electronics &amp; Communication Engineering (ECE) deals with electronic circuits, communication systems, embedded systems, signal processing, IoT, and wireless technologies.</t>
+  </si>
+  <si>
+    <t>What is Electrical &amp; Electronics Engineering?</t>
+  </si>
+  <si>
+    <t>Electrical &amp; Electronics Engineering (EEE) focuses on electrical machines, power systems, control systems, power electronics, and renewable energy.</t>
+  </si>
+  <si>
+    <t>What is Electronics Engineering (VLSI Design)?</t>
+  </si>
+  <si>
+    <t>VLSI Engineering focuses on semiconductor chip design, integrated circuits, embedded systems, and hardware design.</t>
+  </si>
+  <si>
+    <t>What is Electronics &amp; Biomedical Engineering?</t>
+  </si>
+  <si>
+    <t>Electronics &amp; Biomedical Engineering combines electronics with healthcare technology, medical instrumentation, biomedical devices, and diagnostics.</t>
+  </si>
+  <si>
+    <t>What is Mechanical Engineering?</t>
+  </si>
+  <si>
+    <t>Mechanical Engineering focuses on manufacturing, thermodynamics, machine design, robotics, automobiles, and industrial engineering.</t>
+  </si>
+  <si>
+    <t>How many seats are available in Computer Science &amp; Engineering?</t>
+  </si>
+  <si>
+    <t>Computer Science &amp; Engineering has an approved intake of 180 seats.</t>
+  </si>
+  <si>
+    <t>How many seats are available in Electronics &amp; Communication?</t>
+  </si>
+  <si>
+    <t>Electronics &amp; Communication has an approved intake of 120 seats.</t>
+  </si>
+  <si>
+    <t>How many seats are available in Computer Science and Business Systems?</t>
+  </si>
+  <si>
+    <t>Computer Science and Business Systems has an approved intake of 60 seats.</t>
+  </si>
+  <si>
+    <t>How many seats are available in Electrical &amp; Electronics?</t>
+  </si>
+  <si>
+    <t>Electrical &amp; Electronics has an approved intake of 60 seats.</t>
+  </si>
+  <si>
+    <t>How many seats are available in Electronics Engineering (VLSI Design)?</t>
+  </si>
+  <si>
+    <t>Electronics Engineering (VLSI Design) has an approved intake of 60 seats.</t>
+  </si>
+  <si>
+    <t>How many seats are available in Electronics &amp; Biomedical Engineering?</t>
+  </si>
+  <si>
+    <t>Electronics &amp; Biomedical Engineering has an approved intake of 60 seats.</t>
+  </si>
+  <si>
+    <t>How many seats are available in Mechanical Engineering?</t>
+  </si>
+  <si>
+    <t>Mechanical Engineering has an approved intake of 60 seats.</t>
+  </si>
+  <si>
+    <t>How can I get admission to MEC?</t>
+  </si>
+  <si>
+    <t>Admission to Government Model Engineering College is primarily through the KEAM entrance examination conducted by the Commissioner for Entrance Examinations (CEE), Kerala.</t>
+  </si>
+  <si>
+    <t>KEAM is the Kerala Engineering, Architecture, and Medical entrance examination conducted annually for admissions into professional colleges in Kerala.</t>
+  </si>
+  <si>
+    <t>Is KEAM compulsory for engineering admission?</t>
+  </si>
+  <si>
+    <t>Yes. Admission to the regular engineering seats at MEC is primarily based on KEAM rank.</t>
+  </si>
+  <si>
+    <t>Can I get admission without KEAM?</t>
+  </si>
+  <si>
+    <t>Regular B.Tech admission is through KEAM allotment. Management or other admission modes, if available, are governed by the institution and Government regulations.</t>
+  </si>
+  <si>
+    <t>How is branch allotment decided?</t>
+  </si>
+  <si>
+    <t>Branch allotment depends on your KEAM rank, reservation category, seat availability, and your option preferences during the allotment process.</t>
+  </si>
+  <si>
+    <t>What documents are required during admission?</t>
+  </si>
+  <si>
+    <t>Students generally need the KEAM allotment memo, KEAM rank card, SSLC and Plus Two certificates, transfer certificate, conduct certificate, community certificate (if applicable), income certificate (if applicable), and passport-size photographs.</t>
+  </si>
+  <si>
+    <t>What happens after allotment?</t>
+  </si>
+  <si>
+    <t>Students must report to the allotted college within the specified time with all required documents and fee payment to confirm admission.</t>
+  </si>
+  <si>
+    <t>What if I miss the reporting date?</t>
+  </si>
+  <si>
+    <t>Missing the reporting date may result in cancellation of the allotted seat. Students should follow the official CEE schedule carefully.</t>
+  </si>
+  <si>
+    <t>What is spot admission?</t>
+  </si>
+  <si>
+    <t>Spot admission is conducted to fill vacant seats after the regular allotment process according to the rules announced by the authorities.</t>
+  </si>
+  <si>
+    <t>What does the General category mean?</t>
+  </si>
+  <si>
+    <t>General (GN) refers to students who do not belong to any reservation category.</t>
+  </si>
+  <si>
+    <t>What is the Ezhava category?</t>
+  </si>
+  <si>
+    <t>EZ represents the Ezhava reservation category eligible for reservation benefits under Kerala Government rules.</t>
+  </si>
+  <si>
+    <t>What is SC category?</t>
+  </si>
+  <si>
+    <t>SC refers to Scheduled Caste candidates eligible for reservation as per Government norms.</t>
+  </si>
+  <si>
+    <t>What is ST category?</t>
+  </si>
+  <si>
+    <t>ST refers to Scheduled Tribe candidates eligible for reservation benefits.</t>
+  </si>
+  <si>
+    <t>What is MU category?</t>
+  </si>
+  <si>
+    <t>MU represents the Muslim reservation category.</t>
+  </si>
+  <si>
+    <t>What is BH category?</t>
+  </si>
+  <si>
+    <t>BH represents the Other Backward Hindu reservation category.</t>
+  </si>
+  <si>
+    <t>What is VK category?</t>
+  </si>
+  <si>
+    <t>VK represents the Viswakarma reservation category.</t>
+  </si>
+  <si>
+    <t>What is LA category?</t>
+  </si>
+  <si>
+    <t>LA represents the Latin Catholic reservation category.</t>
+  </si>
+  <si>
+    <t>What is KU category?</t>
+  </si>
+  <si>
+    <t>KU represents the Kudumbi reservation category.</t>
+  </si>
+  <si>
+    <t>What is KN category?</t>
+  </si>
+  <si>
+    <t>KN represents the Kusavan reservation category.</t>
+  </si>
+  <si>
+    <t>What is DV category?</t>
+  </si>
+  <si>
+    <t>DV represents the Dheevara reservation category.</t>
+  </si>
+  <si>
+    <t>What is BX category?</t>
+  </si>
+  <si>
+    <t>BX represents the Other Backward Christian reservation category.</t>
+  </si>
+  <si>
+    <t>What is EW category?</t>
+  </si>
+  <si>
+    <t>EW represents the Economically Weaker Sections reservation category.</t>
+  </si>
+  <si>
+    <t>What is MG seat type?</t>
+  </si>
+  <si>
+    <t>MG stands for Merit seat under the Government merit quota.</t>
+  </si>
+  <si>
+    <t>What is SM seat type?</t>
+  </si>
+  <si>
+    <t>SM represents State Merit seats allotted based on KEAM merit.</t>
+  </si>
+  <si>
+    <t>How much is the tuition fee?</t>
+  </si>
+  <si>
+    <t>Tuition fees are decided by the Government and university regulations and may vary each academic year. Students should refer to the latest admission notification.</t>
+  </si>
+  <si>
+    <t>Is hostel fee included in tuition fee?</t>
+  </si>
+  <si>
+    <t>No. Hostel fees are separate from tuition fees.</t>
+  </si>
+  <si>
+    <t>Is there a caution deposit?</t>
+  </si>
+  <si>
+    <t>Yes. Students may be required to pay refundable caution deposits as per college regulations.</t>
+  </si>
+  <si>
+    <t>Can I pay fees online?</t>
+  </si>
+  <si>
+    <t>Fee payment methods are announced during admission and may include online payment facilities.</t>
+  </si>
+  <si>
+    <t>Is hostel facility available?</t>
+  </si>
+  <si>
+    <t>Yes. Hostel facilities are available for eligible students subject to seat availability.</t>
+  </si>
+  <si>
+    <t>Are separate hostels available for boys and girls?</t>
+  </si>
+  <si>
+    <t>Yes. Separate hostel facilities are available for boys and girls.</t>
+  </si>
+  <si>
+    <t>Is hostel admission guaranteed?</t>
+  </si>
+  <si>
+    <t>No. Hostel allotment depends on availability and the hostel admission policy.</t>
+  </si>
+  <si>
+    <t>Does MEC have good placements?</t>
+  </si>
+  <si>
+    <t>Yes. Government Model Engineering College has a strong placement record with several reputed companies visiting the campus every year.</t>
+  </si>
+  <si>
+    <t>Which companies visit MEC?</t>
+  </si>
+  <si>
+    <t>Companies from software, electronics, consulting, analytics, and core engineering sectors regularly participate in campus recruitment.</t>
+  </si>
+  <si>
+    <t>Are internships available?</t>
+  </si>
+  <si>
+    <t>Yes. Many students secure internships through campus drives, faculty guidance, and individual applications.</t>
+  </si>
+  <si>
+    <t>Where is Government Model Engineering College located?</t>
+  </si>
+  <si>
+    <t>Government Model Engineering College is located in Thrikkakara, Kochi, Kerala.</t>
+  </si>
+  <si>
+    <t>Is MEC an autonomous institution?</t>
+  </si>
+  <si>
+    <t>Yes. Government Model Engineering College functions as an autonomous engineering institution under APJ Abdul Kalam Technological University.</t>
+  </si>
+  <si>
+    <t>Which university is MEC affiliated with?</t>
+  </si>
+  <si>
+    <t>MEC is academically affiliated with APJ Abdul Kalam Technological University (KTU).</t>
+  </si>
+  <si>
+    <t>How can I contact the admission office?</t>
+  </si>
+  <si>
+    <t>Students should refer to the official Government Model Engineering College website for the latest admission contact details.</t>
+  </si>
+  <si>
+    <t>Can AdmissionGPT guarantee admission?</t>
+  </si>
+  <si>
+    <t>No. AdmissionGPT provides predictions based on historical admission and cutoff data. Actual admission depends on the official allotment conducted by CEE Kerala.</t>
   </si>
 </sst>
 </file>
@@ -486,7 +714,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D43A6224-62AD-4F23-8F0D-159AF60448C2}">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.28515625" customWidth="1"/>
@@ -501,124 +729,428 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="120" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A44" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A48" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A49" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A50" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+      <c r="A51" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A52" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A53" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+      <c r="A54" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>